<commit_message>
Publish the 장위 13-1 range the review board already marked complete.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/archive/golden/261027/golden_samples_261027.xlsx
+++ b/data/archive/golden/261027/golden_samples_261027.xlsx
@@ -8014,12 +8014,12 @@
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3.91</t>
         </is>
       </c>
       <c r="K53" t="inlineStr"/>
@@ -8603,7 +8603,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3.91</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">

</xml_diff>

<commit_message>
Publish the approved 신길 2 range and the six budget bands.
Hexagon benchmarks now use Golden sheet 84-type dong prices.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/archive/golden/261027/golden_samples_261027.xlsx
+++ b/data/archive/golden/261027/golden_samples_261027.xlsx
@@ -9022,12 +9022,12 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>13.87</t>
+          <t>14</t>
         </is>
       </c>
       <c r="K60" t="inlineStr"/>
@@ -9615,7 +9615,7 @@
       <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr">
         <is>
-          <t>13.87</t>
+          <t>14</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">

</xml_diff>